<commit_message>
#8 Main Board BOM peripheral added
</commit_message>
<xml_diff>
--- a/Design-Files/MotorDriver-v1.0/Deliverables/BOM/Client BOM.xlsx
+++ b/Design-Files/MotorDriver-v1.0/Deliverables/BOM/Client BOM.xlsx
@@ -967,17 +967,16 @@
     <t>2 弹簧天线 2.5dBi Vertical 433MHz - Antennas ROHS</t>
   </si>
   <si>
-    <t xml:space="preserve">VG433SNX39-6W3
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vollgo </t>
-  </si>
-  <si>
-    <t>C718844</t>
-  </si>
-  <si>
     <t>DO NOT Place</t>
+  </si>
+  <si>
+    <t>T14-433M</t>
+  </si>
+  <si>
+    <t>DreamLNK</t>
+  </si>
+  <si>
+    <t>C381188</t>
   </si>
 </sst>
 </file>
@@ -2827,7 +2826,7 @@
         <v>274</v>
       </c>
       <c r="M26" s="62" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -2905,7 +2904,7 @@
         <v>274</v>
       </c>
       <c r="M28" s="62" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -4186,14 +4185,14 @@
       <c r="F62" s="37" t="s">
         <v>277</v>
       </c>
-      <c r="G62" s="55" t="s">
-        <v>313</v>
+      <c r="G62" s="37" t="s">
+        <v>314</v>
       </c>
       <c r="H62" s="37" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I62" s="37" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J62" s="37" t="s">
         <v>274</v>

</xml_diff>